<commit_message>
Major changes to draw logic. Implementation of mat distribution.
</commit_message>
<xml_diff>
--- a/Templates/Poule_5.xlsx
+++ b/Templates/Poule_5.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\winlin\Python\AJDS\Judo-Plus-Sheets\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\winlin\dev\AJDS\Judo-Plus-Sheets\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEDA03E1-E793-42BC-8968-8F4BDE3319B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B62F8E0-00A3-4A61-8813-373052A84734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1 Poule" sheetId="3" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>Nº</t>
   </si>
@@ -97,13 +97,22 @@
   </si>
   <si>
     <t xml:space="preserve">Projecto Judo + </t>
+  </si>
+  <si>
+    <t>Categ:</t>
+  </si>
+  <si>
+    <t>Peso</t>
+  </si>
+  <si>
+    <t>Tapete:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,24 +128,6 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
       <i/>
       <sz val="12"/>
       <color theme="1"/>
@@ -144,39 +135,9 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Palatino Linotype"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
@@ -207,14 +168,42 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Times New Roman"/>
+      <color rgb="FFFF3300"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Palatino Linotype"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Palatino Linotype"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Palatino Linotype"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Palatino Linotype"/>
       <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF3300"/>
-      <name val="Helvetica"/>
-      <family val="2"/>
+      <name val="Palatino Linotype"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Palatino Linotype"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -243,7 +232,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -347,21 +336,6 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -503,27 +477,144 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top/>
       <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -531,157 +622,187 @@
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="após presenças minimas concluidas" xfId="4" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -716,7 +837,7 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>914400</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>192858</xdr:rowOff>
+      <xdr:rowOff>173808</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -765,64 +886,59 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2381</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>4763</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>127254</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>141351</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagem 1">
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="5" name="Straight Connector 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4B9AB2D3-FB0D-4853-3946-011B05B787CF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
-          <a:clrChange>
-            <a:clrFrom>
-              <a:srgbClr val="FEFEFE"/>
-            </a:clrFrom>
-            <a:clrTo>
-              <a:srgbClr val="FEFEFE">
-                <a:alpha val="0"/>
-              </a:srgbClr>
-            </a:clrTo>
-          </a:clrChange>
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5581650" y="5162550"/>
-          <a:ext cx="1517904" cy="646176"/>
+          <a:off x="2726531" y="1852613"/>
+          <a:ext cx="502444" cy="1233487"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom prst="line">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
       </xdr:spPr>
-    </xdr:pic>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1168,430 +1284,465 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:X24"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" customWidth="1"/>
-    <col min="5" max="14" width="5.7109375" customWidth="1"/>
-    <col min="15" max="15" width="8" customWidth="1"/>
-    <col min="16" max="16" width="7.7109375" customWidth="1"/>
-    <col min="19" max="19" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" style="20" customWidth="1"/>
+    <col min="2" max="2" width="22.140625" style="20" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" style="20" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" style="20" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" style="20" customWidth="1"/>
+    <col min="6" max="15" width="5.7109375" style="20" customWidth="1"/>
+    <col min="16" max="16" width="8" style="20" customWidth="1"/>
+    <col min="17" max="17" width="7.7109375" style="20" customWidth="1"/>
+    <col min="18" max="18" width="7" style="20" customWidth="1"/>
+    <col min="19" max="19" width="9.140625" style="20"/>
+    <col min="20" max="20" width="9.5703125" style="20" customWidth="1"/>
+    <col min="21" max="16384" width="9.140625" style="20"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="18" x14ac:dyDescent="0.35">
-      <c r="C1" s="21" t="s">
+    <row r="1" spans="1:24" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D1" s="14" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="18" x14ac:dyDescent="0.35">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="45" t="s">
+    <row r="2" spans="1:24" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-    </row>
-    <row r="3" spans="1:23" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-    </row>
-    <row r="4" spans="1:23" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="54" t="s">
+      <c r="E2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q2" s="25"/>
+      <c r="R2" s="3"/>
+    </row>
+    <row r="3" spans="1:24" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+    </row>
+    <row r="4" spans="1:24" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="L4" s="57"/>
-      <c r="M4" s="60"/>
-      <c r="N4" s="61"/>
-      <c r="O4" s="61"/>
-      <c r="P4" s="61"/>
-      <c r="Q4" s="62"/>
-    </row>
-    <row r="5" spans="1:23" ht="18" x14ac:dyDescent="0.35">
-      <c r="Q5" s="4"/>
-    </row>
-    <row r="7" spans="1:23" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="56" t="s">
+      <c r="J4" s="28"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="33"/>
+      <c r="M4" s="33"/>
+      <c r="N4" s="33"/>
+      <c r="O4" s="34"/>
+      <c r="P4" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="41"/>
+      <c r="R4" s="42"/>
+    </row>
+    <row r="5" spans="1:24" ht="18" x14ac:dyDescent="0.35">
+      <c r="R5" s="3"/>
+    </row>
+    <row r="7" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+      <c r="A7" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="56" t="s">
+      <c r="B7" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="56" t="s">
+      <c r="C7" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="2">
+      <c r="F7" s="43">
         <v>4</v>
       </c>
-      <c r="F7" s="2">
+      <c r="G7" s="43">
         <v>1</v>
       </c>
-      <c r="G7" s="2">
+      <c r="H7" s="43">
         <v>3</v>
       </c>
-      <c r="H7" s="2">
+      <c r="I7" s="43">
         <v>1</v>
       </c>
-      <c r="I7" s="2">
+      <c r="J7" s="43">
         <v>2</v>
       </c>
-      <c r="J7" s="2">
+      <c r="K7" s="43">
         <v>1</v>
       </c>
-      <c r="K7" s="2">
+      <c r="L7" s="43">
         <v>3</v>
       </c>
-      <c r="L7" s="2">
+      <c r="M7" s="43">
         <v>2</v>
       </c>
-      <c r="M7" s="2">
+      <c r="N7" s="43">
         <v>1</v>
       </c>
-      <c r="N7" s="2">
+      <c r="O7" s="43">
         <v>2</v>
       </c>
-      <c r="O7" s="56" t="s">
+      <c r="P7" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="P7" s="56" t="s">
+      <c r="Q7" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="Q7" s="56" t="s">
+      <c r="R7" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="S7" s="4"/>
-      <c r="U7" s="47"/>
-      <c r="V7" s="47"/>
-      <c r="W7" s="47"/>
-    </row>
-    <row r="8" spans="1:23" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="56"/>
-      <c r="B8" s="56"/>
-      <c r="C8" s="56"/>
-      <c r="D8" s="35" t="s">
+      <c r="T7" s="3"/>
+      <c r="V7" s="44"/>
+      <c r="W7" s="44"/>
+      <c r="X7" s="44"/>
+    </row>
+    <row r="8" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+      <c r="A8" s="31"/>
+      <c r="B8" s="31"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="2">
+      <c r="F8" s="43">
         <v>5</v>
       </c>
-      <c r="F8" s="2">
+      <c r="G8" s="43">
         <v>2</v>
       </c>
-      <c r="G8" s="2">
+      <c r="H8" s="43">
         <v>4</v>
       </c>
-      <c r="H8" s="2">
+      <c r="I8" s="43">
         <v>5</v>
       </c>
-      <c r="I8" s="2">
+      <c r="J8" s="43">
         <v>3</v>
       </c>
-      <c r="J8" s="2">
+      <c r="K8" s="43">
         <v>4</v>
       </c>
-      <c r="K8" s="2">
+      <c r="L8" s="43">
         <v>5</v>
       </c>
-      <c r="L8" s="2">
+      <c r="M8" s="43">
         <v>4</v>
       </c>
-      <c r="M8" s="2">
+      <c r="N8" s="43">
         <v>3</v>
       </c>
-      <c r="N8" s="2">
+      <c r="O8" s="43">
         <v>5</v>
       </c>
-      <c r="O8" s="56"/>
-      <c r="P8" s="56"/>
-      <c r="Q8" s="56"/>
-      <c r="S8" s="4"/>
-      <c r="U8" s="46"/>
-      <c r="V8" s="46"/>
-      <c r="W8" s="46"/>
-    </row>
-    <row r="9" spans="1:23" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="29">
+      <c r="P8" s="31"/>
+      <c r="Q8" s="31"/>
+      <c r="R8" s="31"/>
+      <c r="T8" s="3"/>
+      <c r="V8" s="45"/>
+      <c r="W8" s="45"/>
+      <c r="X8" s="45"/>
+    </row>
+    <row r="9" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+      <c r="A9" s="17">
         <v>1</v>
       </c>
-      <c r="B9" s="48"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="48"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="25"/>
-      <c r="K9" s="26"/>
-      <c r="L9" s="26"/>
-      <c r="M9" s="25"/>
-      <c r="N9" s="27"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="S9" s="4"/>
-      <c r="U9" s="46"/>
-      <c r="V9" s="46"/>
-      <c r="W9" s="46"/>
-    </row>
-    <row r="10" spans="1:23" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="29">
+      <c r="B9" s="46"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="50"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="52"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="52"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="52"/>
+      <c r="O9" s="53"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="T9" s="3"/>
+      <c r="V9" s="45"/>
+      <c r="W9" s="45"/>
+      <c r="X9" s="45"/>
+    </row>
+    <row r="10" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+      <c r="A10" s="17">
         <v>2</v>
       </c>
-      <c r="B10" s="48"/>
-      <c r="C10" s="48"/>
-      <c r="D10" s="48"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="25"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="25"/>
-      <c r="M10" s="26"/>
-      <c r="N10" s="25"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="3"/>
-      <c r="S10" s="4"/>
-      <c r="U10" s="46"/>
-      <c r="V10" s="46"/>
-      <c r="W10" s="46"/>
-    </row>
-    <row r="11" spans="1:23" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="29">
+      <c r="B10" s="46"/>
+      <c r="C10" s="46"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="54"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="50"/>
+      <c r="H10" s="51"/>
+      <c r="I10" s="51"/>
+      <c r="J10" s="52"/>
+      <c r="K10" s="53"/>
+      <c r="L10" s="51"/>
+      <c r="M10" s="52"/>
+      <c r="N10" s="51"/>
+      <c r="O10" s="52"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="T10" s="3"/>
+      <c r="V10" s="45"/>
+      <c r="W10" s="45"/>
+      <c r="X10" s="45"/>
+    </row>
+    <row r="11" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+      <c r="A11" s="17">
         <v>3</v>
       </c>
-      <c r="B11" s="37"/>
-      <c r="C11" s="51"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="27"/>
-      <c r="M11" s="25"/>
-      <c r="N11" s="27"/>
-      <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
-      <c r="Q11" s="3"/>
-      <c r="S11" s="4"/>
-      <c r="U11" s="46"/>
-      <c r="V11" s="46"/>
-      <c r="W11" s="46"/>
-    </row>
-    <row r="12" spans="1:23" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="29">
+      <c r="B11" s="55"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="56"/>
+      <c r="E11" s="54"/>
+      <c r="F11" s="57"/>
+      <c r="G11" s="58"/>
+      <c r="H11" s="52"/>
+      <c r="I11" s="51"/>
+      <c r="J11" s="52"/>
+      <c r="K11" s="53"/>
+      <c r="L11" s="52"/>
+      <c r="M11" s="53"/>
+      <c r="N11" s="52"/>
+      <c r="O11" s="53"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+      <c r="T11" s="3"/>
+      <c r="V11" s="45"/>
+      <c r="W11" s="45"/>
+      <c r="X11" s="45"/>
+    </row>
+    <row r="12" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+      <c r="A12" s="17">
         <v>4</v>
       </c>
-      <c r="B12" s="52"/>
-      <c r="C12" s="53"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="36"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="27"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="26"/>
-      <c r="N12" s="27"/>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="3"/>
-      <c r="S12" s="4"/>
-      <c r="U12" s="19"/>
-    </row>
-    <row r="13" spans="1:23" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="3">
+      <c r="B12" s="59"/>
+      <c r="C12" s="59"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="54"/>
+      <c r="F12" s="60"/>
+      <c r="G12" s="58"/>
+      <c r="H12" s="52"/>
+      <c r="I12" s="51"/>
+      <c r="J12" s="51"/>
+      <c r="K12" s="52"/>
+      <c r="L12" s="53"/>
+      <c r="M12" s="52"/>
+      <c r="N12" s="51"/>
+      <c r="O12" s="53"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="T12" s="3"/>
+      <c r="V12" s="61"/>
+    </row>
+    <row r="13" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+      <c r="A13" s="2">
         <v>5</v>
       </c>
-      <c r="B13" s="50"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="26"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="26"/>
-      <c r="M13" s="26"/>
-      <c r="N13" s="25"/>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="3"/>
-      <c r="S13" s="4"/>
-      <c r="U13" s="47"/>
-      <c r="V13" s="47"/>
-      <c r="W13" s="47"/>
-    </row>
-    <row r="14" spans="1:23" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="S14" s="4"/>
-      <c r="U14" s="46"/>
-      <c r="V14" s="46"/>
-      <c r="W14" s="46"/>
-    </row>
-    <row r="15" spans="1:23" ht="20.25" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="I15" s="38"/>
-      <c r="K15" s="20"/>
-      <c r="S15" s="4"/>
-      <c r="U15" s="46"/>
-      <c r="V15" s="46"/>
-      <c r="W15" s="46"/>
-    </row>
-    <row r="16" spans="1:23" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="54" t="s">
+      <c r="B13" s="62"/>
+      <c r="C13" s="62"/>
+      <c r="D13" s="63"/>
+      <c r="E13" s="64"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="51"/>
+      <c r="H13" s="51"/>
+      <c r="I13" s="52"/>
+      <c r="J13" s="51"/>
+      <c r="K13" s="51"/>
+      <c r="L13" s="52"/>
+      <c r="M13" s="51"/>
+      <c r="N13" s="51"/>
+      <c r="O13" s="52"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
+      <c r="T13" s="3"/>
+      <c r="V13" s="44"/>
+      <c r="W13" s="44"/>
+      <c r="X13" s="44"/>
+    </row>
+    <row r="14" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+      <c r="T14" s="3"/>
+      <c r="V14" s="45"/>
+      <c r="W14" s="45"/>
+      <c r="X14" s="45"/>
+    </row>
+    <row r="15" spans="1:24" ht="21.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="J15" s="19"/>
+      <c r="L15" s="13"/>
+      <c r="T15" s="3"/>
+      <c r="V15" s="45"/>
+      <c r="W15" s="45"/>
+      <c r="X15" s="45"/>
+    </row>
+    <row r="16" spans="1:24" ht="23.25" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="55"/>
-      <c r="C16" s="11" t="s">
+      <c r="B16" s="27"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="4"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="41"/>
-      <c r="K16" s="39"/>
-      <c r="S16" s="4"/>
-      <c r="U16" s="46"/>
-      <c r="V16" s="46"/>
-      <c r="W16" s="46"/>
-    </row>
-    <row r="17" spans="1:23" ht="20.25" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="6" t="s">
+      <c r="E16" s="3"/>
+      <c r="H16" s="21"/>
+      <c r="I16" s="65"/>
+      <c r="T16" s="3"/>
+      <c r="V16" s="45"/>
+      <c r="W16" s="45"/>
+      <c r="X16" s="45"/>
+    </row>
+    <row r="17" spans="1:24" ht="21.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="30"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="4"/>
-      <c r="I17" s="58" t="s">
+      <c r="B17" s="66"/>
+      <c r="C17" s="67"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="3"/>
+      <c r="J17" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="J17" s="59"/>
-      <c r="K17" s="59"/>
-      <c r="L17" s="42"/>
-      <c r="S17" s="4"/>
-      <c r="U17" s="46"/>
-      <c r="V17" s="46"/>
-      <c r="W17" s="46"/>
-    </row>
-    <row r="18" spans="1:23" ht="18" x14ac:dyDescent="0.35">
-      <c r="A18" s="7" t="s">
+      <c r="K17" s="30"/>
+      <c r="L17" s="30"/>
+      <c r="M17" s="68"/>
+      <c r="T17" s="3"/>
+      <c r="V17" s="45"/>
+      <c r="W17" s="45"/>
+      <c r="X17" s="45"/>
+    </row>
+    <row r="18" spans="1:24" ht="18" x14ac:dyDescent="0.35">
+      <c r="A18" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="22"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="4"/>
-      <c r="S18" s="4"/>
-    </row>
-    <row r="19" spans="1:23" ht="18" x14ac:dyDescent="0.35">
-      <c r="A19" s="7" t="s">
+      <c r="B18" s="37"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="3"/>
+      <c r="T18" s="3"/>
+    </row>
+    <row r="19" spans="1:24" ht="18" x14ac:dyDescent="0.35">
+      <c r="A19" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="4"/>
-      <c r="S19" s="4"/>
-    </row>
-    <row r="20" spans="1:23" ht="18" x14ac:dyDescent="0.35">
-      <c r="A20" s="7" t="s">
+      <c r="B19" s="37"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="3"/>
+      <c r="T19" s="3"/>
+    </row>
+    <row r="20" spans="1:24" ht="18" x14ac:dyDescent="0.35">
+      <c r="A20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="22"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="4"/>
-      <c r="S20" s="4"/>
-    </row>
-    <row r="21" spans="1:23" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="23" t="s">
+      <c r="B20" s="37"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="3"/>
+      <c r="T20" s="3"/>
+    </row>
+    <row r="21" spans="1:24" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="4"/>
-      <c r="S21" s="4"/>
-    </row>
-    <row r="23" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="1:23" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B24" s="12" t="s">
+      <c r="B21" s="39"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="3"/>
+      <c r="T21" s="3"/>
+    </row>
+    <row r="23" spans="1:24" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="24" spans="1:24" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B24" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C24" s="13"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="G24" s="15" t="s">
+      <c r="C24" s="10"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="3"/>
+      <c r="H24" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="17"/>
-      <c r="K24" s="18"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
-      <c r="N24" s="5"/>
-      <c r="O24" s="5"/>
+      <c r="I24" s="69"/>
+      <c r="J24" s="69"/>
+      <c r="K24" s="70"/>
+      <c r="L24" s="71"/>
+      <c r="M24" s="72"/>
+      <c r="N24" s="72"/>
+      <c r="O24" s="72"/>
+      <c r="P24" s="72"/>
+      <c r="Q24" s="72"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="S7:S18">
-    <sortCondition ref="S7"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="T7:T18">
+    <sortCondition ref="T7"/>
   </sortState>
-  <mergeCells count="10">
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="P7:P8"/>
+  <mergeCells count="18">
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="J17:L17"/>
     <mergeCell ref="Q7:Q8"/>
-    <mergeCell ref="M4:Q4"/>
-    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="R7:R8"/>
+    <mergeCell ref="K4:O4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="Q4:R4"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="B7:B8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="P7:P8"/>
+    <mergeCell ref="E9:E13"/>
     <mergeCell ref="C7:C8"/>
-    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="B17:C17"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>